<commit_message>
added initial test scenarios in xlsx
</commit_message>
<xml_diff>
--- a/SauceDemo Testings.xlsx
+++ b/SauceDemo Testings.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\me\Documents\SauceDemo-Website-Testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A2971C8F-06A0-4017-B02B-A8E38F0A822F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7848046D-A00A-42EB-B279-1B2005B07D2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{51F5D2F4-61C3-467D-978D-E0E7425A5E44}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Test Plan" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,9 +39,53 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+  <si>
+    <t>l</t>
+  </si>
+  <si>
+    <t>Login Page</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>Fail</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
+    <t>Pass or Fail</t>
+  </si>
+  <si>
+    <t>Note</t>
+  </si>
+  <si>
+    <t>Logging In 'standard_user" Account With Correct Credentials</t>
+  </si>
+  <si>
+    <t>Logging In 'locked_out_user" Account With Correct Credentials</t>
+  </si>
+  <si>
+    <t>Logging In 'problem_user" Account With Correct Credentials</t>
+  </si>
+  <si>
+    <t>Logging In 'performance_glitch_user" Account With Correct Credentials</t>
+  </si>
+  <si>
+    <t>Logging In 'error_user" Account With Correct Credentials</t>
+  </si>
+  <si>
+    <t>Logging In 'visual_user" Account With Correct Credentials</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -48,13 +93,33 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -69,8 +134,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -405,9 +476,95 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A73C241-6A9F-4B50-AEF9-963BB7365548}">
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.140625" customWidth="1"/>
+    <col min="3" max="3" width="62.42578125" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" customWidth="1"/>
+    <col min="5" max="5" width="76.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="1"/>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="2"/>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C3" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C4" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C9" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="C10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="C4:E4"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D410000-CF9A-46E6-A54E-7E65225F56B3}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>